<commit_message>
Update second FYP meeting materials and project documentation
</commit_message>
<xml_diff>
--- a/materials/FYP文献参考.xlsx
+++ b/materials/FYP文献参考.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>序号</t>
   </si>
@@ -60,6 +60,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>1，游戏被用作促进互动的工具，引导参观者理解复杂的概念，同时根据每个人的需求进行</t>
     </r>
     <r>
@@ -146,6 +153,14 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="6"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>1.</t>
     </r>
     <r>
@@ -179,6 +194,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>1，</t>
     </r>
     <r>
@@ -206,6 +228,14 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="6"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>1.</t>
     </r>
     <r>
@@ -321,6 +351,14 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="6"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>1，</t>
     </r>
     <r>
@@ -375,6 +413,310 @@
       </rPr>
       <t xml:space="preserve">
 通过旅游业来寻找非凡的事物是一种社会建构的行为。大众媒体通过摄影的方式创造了人们对外国地方的视觉消费的社会需求（Urry, 2002）。照片改变了并放大了我们对值得观赏事物的认知，而摄影最宏大的成果就是以一种将体验转化为图像、一种纪念品的方式来验证经历的存在（Sontag, 1977）。许多旅游景点都被设计成能够提供良好的拍照机会，并呈现特定的视角（Jansson, 2007）。拥有一张自己在地标前的照片，就相当于“曾经到过那里”的证明（Stylianou-Lambert, 2012）。游客通过选择、构图以及在旅行期间和旅行后创造的内容来体验这些地方（Urry, 1990, 2002）。正如 Larsen（2008）所指出的，数字化带来的旅行摄影方式的变革……借助互联网、电子邮件和手机等新媒体手段传播的旅行图片，彻底改变了旅行行业中的图片传播方式，也影响了游客的旅游体验。在社交媒体的时代，游客不仅通过自己的眼睛观察世界，还借助想象中的观众们的视角来感知世界（Liu 等人，2023 年；Lo 等人，2011 年；Mostafanezhad 和 Norum，2018 年）。</t>
+    </r>
+  </si>
+  <si>
+    <t>https://dl.acm.org/doi/full/10.1145/3772318.3791068</t>
+  </si>
+  <si>
+    <t>LLM-based Embodied Conversational Agent for Reducing Foreign Language Speaking Anxiety in Social VR</t>
+  </si>
+  <si>
+    <r>
+      <t>1，搭载 OpenAI 的实时 API（音频转音频）通</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>双向流通WebSocket</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>去除tts和stt转换过程</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>，最大限度的降低延迟，模拟真实的英语交流</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">In this iteration, we used OpenAI’s Realtime API (audio to audio) [50] to support bidirectional interaction with reduced latency through a persistent WebSocket session [51]. This removes the need for the text-to-speech (TTS) and speech-to-text (STT) cycle and the need for a separate short-term memory module. We retain only a lightweight long-term memory store to track user progress across sessions. The overall ELLMA-T architecture is shown in Figure 4.
+At the start of each WebSocket session, the system loads a prompt file (see details in Appendix E) that defines user background, agent persona, response tone, role behavior, scene context, and workflow logic. Although the maximum duration of a Realtime session is 30 minutes [51], our pilot tests showed that the system maintained high-quality performance for about 15 minutes of continuous dialogue, after which conversational quality gradually declined. For that reason, we limited each scenario to 15 minutes.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>在本次迭代中，我们使用了 OpenAI 的实时 API（音频到音频）[50]，通过持久化的 WebSocket 会话实现双向交互并降低延迟[51]。这消除了文本转语音（TTS）和语音转文本（STT）的循环，也无需单独的短期记忆模块。我们仅保留一个轻量级的长期记忆存储，用于跟踪用户在不同会话中的进展。整体 ELLMA-T 架构如图 4 所示。
+每个 WebSocket 会话开始时，系统会加载一个提示文件（详见附录 E），该文件定义了用户的背景信息、角色设定、回应语气、行为方式、场景情境以及工作流程逻辑。尽管实时会话的最大持续时间是 30 分钟[51]，但我们的试点测试表明，系统在连续对话约 15 分钟后仍能保持高质量表现，之后对话质量逐渐下降。因此，我们将每个场景的持续时间限制为 15 分钟。</t>
+    </r>
+  </si>
+  <si>
+    <t>https://dl.acm.org/doi/10.1145/3706599.3720162#sec-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ConversAR: Exploring Embodied LLM-Powered Group Conversations in Augmented Reality for Second Language Learners
+</t>
+  </si>
+  <si>
+    <r>
+      <t>1，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>单一管道传递websocket，轮流交替传递信息</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>，预先处理下一段信息，降低延迟，</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">We utilize the OpenAI Audio API’s speech-to-text (STT) and text-to-speech (TTS) modules to handle all voice-based inputs and outputs. Users interact with the agents by holding the trigger button on the right Meta Quest Touch controller and speaking in the target language. Although we considered voice-based triggers, our pilot studies suggested that the button interaction was intuitive and felt familiar to using a walkie-talkie. This approach also supports mid-speech pausing, addressing a limitation of fully voice-based conversational systems that struggle to distinguish whether the user intends to stop speaking or is pausing to think [40]. When the user lets go of the trigger, their speech is saved as an mp3 file that is passed through the "whisper-1" model and is finally returned as text output to prompt agent responses. Agent responses are verbalized via the Audio API and displayed in live caption windows underneath each agent, following accessible caption placement recommendations from prior AR research [25].
+The STT module exhibited high accuracy but occasionally auto-corrected user speech inputs in ambiguous cases (e.g., unclear pronunciation, filler words, incorrect tense usage) to maintain grammatical consistency, which pilot testers found helpful for error recognition. The TTS model also performed well, with pronunciation evaluated as natural and correct by a native Spanish-speaking researcher. However, there was an observable delay when transitioning from STT to TTS. While this delay was imperceptible during agent-to-agent interactions where the next utterance is preemptively generated and stored, STT user inputs consistently resulted in a 1-2 second pause before TTS agent responses. This delay scaled proportionally with longer, more complex speech inputs, however, did not impede the experience across pilot and study sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>我们使用 OpenAI 音频 API 的语音转文字（STT）和文字转语音（TTS）模块来处理所有基于语音的输入和输出。用户通过按住 Meta Quest Touch 控制器右侧的触发按钮，并以目标语言进行说话，与智能体交互。尽管我们考虑了语音触发方式，但试点研究表明，这种按钮操作直观且类似于使用对讲机，用户感觉熟悉。该方法还支持在说话过程中暂停，解决了完全基于语音的对话系统的一个局限性：即难以判断用户是想停止说话，还是在暂停思考[40]。当用户松开触发按钮时，其语音会被保存为 mp3 文件，经由“whisper-1”模型处理后，最终以文本形式返回，用于提示智能体作出回应。智能体的回复将通过音频 API 转为语音，并根据以往 AR 研究中提出的可访问字幕布局建议[25]，显示在每个智能体下方的实时字幕窗口中。
+STT模块表现出高准确性，但在语义模糊的情况下（例如发音不清、填充词、时态使用错误）会自动修正用户语音输入，以保持语法一致性，试点测试者认为这有助于识别错误。TTS模型也表现良好，其发音被一名母语为西班牙语的研究人员评价为自然且正确。然而，在从STT切换到TTS的过程中存在明显的延迟。虽然在人与人交互中，由于下一句话语会被预先生成并存储，这种延迟几乎察觉不到，但STT用户的输入始终会导致TTS代理响应前出现1至2秒的暂停。该延迟随着语音输入更长、更复杂而按比例增加，但并未影响试点和研究阶段的整体体验。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">A gpt-4o powered "Moderator LLM" transitions the conversation between agent-speaking and user-speaking states. During the agent-speaking state, the conversation oscillates between the two agents indefinitely. The agents direct responses to each other and the user, but ultimately the user decides when to reply or interject. For example, one agent may ask the user a direct question, but if they do not respond during a defined conversational gap, the other agent will respond instead. This approach was designed to prepare users for conversation dynamics in which a delayed response or lack of contribution leads to other interlocutors continuing the discussion. This is a common reality for L2 learners, especially when engaging in group conversations dominated by more proficient or native speakers [48]. Through pilot studies, we determined an optimal gap of 3 seconds between each agent-generated response. Users can transition to the user-speaking state at any time by holding the right controller trigger, initiating STT. After the user responds, the "Moderator LLM" analyzes the conversation history to select the most appropriate responding agent (Fig. 3). This setup allows users to continue the activity indefinitely.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">由GPT-4o驱动的“主持人LLM”在代理发言和用户发言之间进行对话切换。在代理发言状态下，对话会无限循环地在两个代理之间交替。代理们相互之间以及与用户之间发出回应，但最终由用户决定何时回复或插话。例如，一个代理可能会向用户提出直接问题，但如果用户在规定的对话间隔内没有回应，另一个代理将代替其作出回应。该设计旨在帮助用户适应一种对话动态：延迟回应或未参与讨论时，其他对话者会继续推进对话。这种现象在第二语言学习者中十分常见，尤其是在以更熟练或母语者为主的小组对话中[48]。通过试点研究，我们确定了每个代理生成响应之间最佳的3秒间隔。用户可随时通过按住正确的控制器触发键来启动语音转文字（STT），从而进入用户发言状态。用户回应后，“主持人LLM”会分析对话历史，选择最合适的回应代理（图3）。该设置使用户能够无限期地继续活动。  </t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s40494-025-01889-3</t>
+  </si>
+  <si>
+    <t>Design and evaluation of touch and touchless interfaces for interactive digital heritage experiences
+为互动数字文化遗产体验设计和评估有触感和无触感的交互界面。</t>
+  </si>
+  <si>
+    <t>1，滑动、选择、平移、旋转、放大和缩小等。我们将这些操作动作整合起来，从而设计出更加丰富的交互式手势，为触摸和手势界面提供了必要的操作技巧。
+2，我们使用的技术包括使用 Blender 软件构建 3D 模型 45 （图 2a），通过 Procreate 软件进行数字绘画以创建纹理 46 （图 2b），最后在 Unity 游戏中将纹理应用到模型上
+3，基于 Unity 引擎开发了一个适用于 iOS 系统的虚拟平台，该平台可以在 iPad 上运行，用户可以通过触摸屏来体验虚拟博物馆展览。
+4，触摸界面的操作（如图 3c 所示）与滑动操作（如图 3a 所示）类似，但区别在于用户需要将手指持续接触屏幕（OHPM），这样物体就会跟随手指的移动轨迹。当手指离开屏幕时，物体就会停止移动。
+5，在触摸界面中，物体的操作方式与平移操作相同（OHPM），而物体旋转的速度和角度则由手指在屏幕上移动的速度和幅度来决定。
+6，在触摸界面中，用户可以通过同时触摸屏幕上的两个手指来实现缩放操作：分开手指可以缩小物体；合拢手指则可以放大物体。缩放的幅度取决于两个手指之间的距离。</t>
+  </si>
+  <si>
+    <r>
+      <t>1，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Traditional methods of displaying artworks often limit direct interaction due to the risk of damage, while some artworks are also fragile or immobile preventing viewers from understanding and experiencing all aspects of the artwork1. In contrast, digital heritage provides a dynamic and immersive platform that enables viewers to explore, manipulate, and engage with digital artifacts in previously unattainable ways. Interactivity in this context is not merely a supplementary feature but a critical component that deepens visitors’ understanding and appreciation of cultural objects. Through the use of interactive technologies, cultural heritage becomes more accessible and engaging, offering contextual information, multidimensional perspectives, and narrative-rich experiences. This enriched engagement fosters a stronger connection between audiences and cultural heritage, thereby enhancing both cultural communication and emotional resonance.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">传统的方式往往因为担心损坏而限制观众的直接互动，而有些艺术品本身又过于脆弱或无法移动，这使得观众无法全面理解或体验这些艺术品。相比之下，数字遗产提供了一个动态且沉浸式平台，让观众能够以以往无法实现的方式探索、操作并与数字作品进行互动。在这种情况下，互动性不仅仅是一个附加功能，而是一个能够加深观众理解与欣赏的重要元素。文化对象的数字化呈现。通过运用互动技术，文化遗产变得更加易于获取且引人入胜。这种数字化形式能够提供上下文信息、多维度视角，以及充满叙事性的体验。这种增强的互动方式有助于加深观众与文化遗产之间的联系，从而提升文化传播的效果以及情感共鸣的效果。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="5"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The hand gesture for interaction is specifically designed for guided tours, interactive experiences and entertainment in virtual museums. Ideally, the interaction of a virtual environment should be consistent with the conceptual model in the mind of each user without any explanation19. Manghisi et al.18 used a cognitive load approach to elicit a set of natural gesture interaction techniques for experiencing cultural heritage interfaces, which are consistent with users’ daily behavioral patterns and are scientifically valid. Therefore, we referred to the gestures with lower cognitive load proposed in18, along with the necessary actions for experiencing virtual tours, including swipe, selection, translation, rotation, zoom-in, and zoom-out. We integrated and supplemented these actions to design interactive gestures, preparing essential operational techniques for touch and gesture interfaces. Figure 3 presents and briefly describes all the gestures proposed for performing these six actions, which will be further explained in the following sections.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+这种用于交互的手势设计，是专门为导览、互动体验以及虚拟博物馆中的娱乐功能而制定的。理想情况下，虚拟环境的互动方式应该与每个用户心中的概念模型保持一致，而无需任何额外的解释。Manghisi 等人提出了一种认知负荷的方法，以引出一系列自然的手势交互技巧，这些技巧能够符合用户的日常行为模式，并且具有科学上的有效性。因此，我们借鉴了 18 中提出的低认知负荷手势方式，同时结合了一些必要的操作动作，比如滑动、选择、平移、旋转、放大和缩小等。我们将这些操作动作整合起来，从而设计出更加丰富的交互式手势，为触摸和手势界面提供了必要的操作技巧。图 3 展示了用于执行这六种动作的所有手势，并简要描述了这些手势的具体操作方式。这些手势将在后续章节中进一步详细说明。</t>
+    </r>
+  </si>
+  <si>
+    <t>https://doi.org/10.1145/3700881</t>
+  </si>
+  <si>
+    <t>HeritageSite AR: Design and Evaluation of a Mobile Augmented Reality Exploration Game for a Chinese Heritage Site
+文化遗产遗址 AR：为中国文化遗产遗址设计并评估一款移动增强现实探索游戏</t>
+  </si>
+  <si>
+    <t>1，Qualcomm 公司的 Vuforia 软件开发工具包（版本 9.8.31）。Vuforia 提供了多种功能支持，包括 2D 和 3D 图像目标识别，以及无标记目标跟踪和多目标跟踪功能。该工具与 iOS 和 Android 平台的原生开发方式兼容，并且能够与 Unity 游戏引擎无缝集成，从而便于 AR 应用的开发。
+2，简化了 3D 模型的设计，使其能够在低性能的移动设备上运行，而不会造成明显的性能下降。此外，我们还评估了用于 AR 的图像目标的大小和质量，确保其大小不超过 2MB，并且识别准确率达到三星级以上。</t>
+  </si>
+  <si>
+    <r>
+      <t>1，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>For the AR game development, we used Unity (version 2020 3.33f1c2) and the Vuforia3 Software Development Kit from Qualcomm (version 9.8.31). Vuforia offers support for a range of features, including 2D and 3D image target recognition, as well as markerless and multi-target tracking. It is compatible with native development for both iOS and Android platforms and seamlessly integrates with the Unity game engine for AR application development. Several key factors were considered in the AR game development and testing, including the available resources, hardware requirements, and the usability of the implemented game design. For example, we made some efforts to simplify the 3D models so that they could be used in low-end mobile devices without causing noticeable delays. We also assessed the size and quality of the image targets used for AR, ensuring that they were under 2 MB in size and achieved a minimum recognition rating of three stars (out of a total of five). To test the quality of image targets in use, we connected to a Redmi Note 11T Pro+ smartphone using the USB debugging tool (see Figure 8). During testing, we addressed some issues caused by the overlapping positions of the models on the mobile interface and issues related to lighting and rendering effects.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="6"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>在 AR 游戏开发过程中，我们使用了 Unity 引擎（版本 2020 3.33f1c2）以及 Qualcomm 公司的 Vuforia 软件开发工具包（版本 9.8.31）。Vuforia 提供了多种功能支持，包括 2D 和 3D 图像目标识别，以及无标记目标跟踪和多目标跟踪功能。该工具与 iOS 和 Android 平台的原生开发方式兼容，并且能够与 Unity 游戏引擎无缝集成，从而便于 AR 应用的开发。在 AR 游戏开发及测试过程中，我们考虑了多个关键因素，如可用资源、硬件要求以及所实现游戏设计的可用性。例如，我们努力简化了 3D 模型的设计，使其能够在低性能的移动设备上运行，而不会造成明显的性能下降。此外，我们还评估了用于 AR 的图像目标的大小和质量，确保其大小不超过 2MB，并且识别准确率达到三星级以上。在总共五个样本中，我们选择了其中一个进行测试。为了检验实际使用中的图像目标质量，我们连接了 Redmi Note 11T Pro+智能手机，并使用 USB 调试工具进行了测试（参见图 8）。在测试过程中，我们解决了由于模型在移动设备界面上位置重叠导致的一些问题，以及与照明和渲染效果相关的问题。</t>
     </r>
   </si>
 </sst>
@@ -388,7 +730,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -556,8 +898,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="9"/>
+      <color theme="5"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -572,7 +915,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="5"/>
+      <color rgb="FFFFC000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1040,7 +1390,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1079,6 +1429,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1394,7 +1747,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U22"/>
+  <dimension ref="A1:U50"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <sheetData>
     <row r="1" spans="1:21">
@@ -1943,8 +2296,692 @@
       <c r="T22" s="12"/>
       <c r="U22" s="12"/>
     </row>
+    <row r="23" spans="1:21">
+      <c r="A23" s="6">
+        <v>4</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="8"/>
+      <c r="D23" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="9"/>
+      <c r="F23" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="12"/>
+      <c r="Q23" s="12"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="12"/>
+      <c r="T23" s="12"/>
+      <c r="U23" s="12"/>
+    </row>
+    <row r="24" spans="1:21">
+      <c r="A24" s="6"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="12"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="12"/>
+      <c r="T24" s="12"/>
+      <c r="U24" s="12"/>
+    </row>
+    <row r="25" spans="1:21">
+      <c r="A25" s="6"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="12"/>
+      <c r="P25" s="12"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
+      <c r="S25" s="12"/>
+      <c r="T25" s="12"/>
+      <c r="U25" s="12"/>
+    </row>
+    <row r="26" spans="1:21">
+      <c r="A26" s="6"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="12"/>
+      <c r="P26" s="12"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
+      <c r="S26" s="12"/>
+      <c r="T26" s="12"/>
+      <c r="U26" s="12"/>
+    </row>
+    <row r="27" spans="1:21">
+      <c r="A27" s="6"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
+      <c r="O27" s="12"/>
+      <c r="P27" s="12"/>
+      <c r="Q27" s="12"/>
+      <c r="R27" s="12"/>
+      <c r="S27" s="12"/>
+      <c r="T27" s="12"/>
+      <c r="U27" s="12"/>
+    </row>
+    <row r="28" spans="1:21">
+      <c r="A28" s="6"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="12"/>
+      <c r="P28" s="12"/>
+      <c r="Q28" s="12"/>
+      <c r="R28" s="12"/>
+      <c r="S28" s="12"/>
+      <c r="T28" s="12"/>
+      <c r="U28" s="12"/>
+    </row>
+    <row r="29" spans="1:21">
+      <c r="A29" s="6"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12"/>
+      <c r="O29" s="12"/>
+      <c r="P29" s="12"/>
+      <c r="Q29" s="12"/>
+      <c r="R29" s="12"/>
+      <c r="S29" s="12"/>
+      <c r="T29" s="12"/>
+      <c r="U29" s="12"/>
+    </row>
+    <row r="30" spans="1:21">
+      <c r="A30" s="6">
+        <v>5</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="8"/>
+      <c r="D30" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" s="9"/>
+      <c r="F30" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="M30" s="12"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="12"/>
+      <c r="P30" s="12"/>
+      <c r="Q30" s="12"/>
+      <c r="R30" s="12"/>
+      <c r="S30" s="12"/>
+      <c r="T30" s="12"/>
+      <c r="U30" s="12"/>
+    </row>
+    <row r="31" spans="1:21">
+      <c r="A31" s="6"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
+      <c r="O31" s="12"/>
+      <c r="P31" s="12"/>
+      <c r="Q31" s="12"/>
+      <c r="R31" s="12"/>
+      <c r="S31" s="12"/>
+      <c r="T31" s="12"/>
+      <c r="U31" s="12"/>
+    </row>
+    <row r="32" spans="1:21">
+      <c r="A32" s="6"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="12"/>
+      <c r="P32" s="12"/>
+      <c r="Q32" s="12"/>
+      <c r="R32" s="12"/>
+      <c r="S32" s="12"/>
+      <c r="T32" s="12"/>
+      <c r="U32" s="12"/>
+    </row>
+    <row r="33" spans="1:21">
+      <c r="A33" s="6"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="12"/>
+      <c r="M33" s="12"/>
+      <c r="N33" s="12"/>
+      <c r="O33" s="12"/>
+      <c r="P33" s="12"/>
+      <c r="Q33" s="12"/>
+      <c r="R33" s="12"/>
+      <c r="S33" s="12"/>
+      <c r="T33" s="12"/>
+      <c r="U33" s="12"/>
+    </row>
+    <row r="34" spans="1:21">
+      <c r="A34" s="6"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+      <c r="P34" s="12"/>
+      <c r="Q34" s="12"/>
+      <c r="R34" s="12"/>
+      <c r="S34" s="12"/>
+      <c r="T34" s="12"/>
+      <c r="U34" s="12"/>
+    </row>
+    <row r="35" spans="1:21">
+      <c r="A35" s="6"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="10"/>
+      <c r="L35" s="12"/>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12"/>
+      <c r="O35" s="12"/>
+      <c r="P35" s="12"/>
+      <c r="Q35" s="12"/>
+      <c r="R35" s="12"/>
+      <c r="S35" s="12"/>
+      <c r="T35" s="12"/>
+      <c r="U35" s="12"/>
+    </row>
+    <row r="36" spans="1:21">
+      <c r="A36" s="6"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="12"/>
+      <c r="M36" s="12"/>
+      <c r="N36" s="12"/>
+      <c r="O36" s="12"/>
+      <c r="P36" s="12"/>
+      <c r="Q36" s="12"/>
+      <c r="R36" s="12"/>
+      <c r="S36" s="12"/>
+      <c r="T36" s="12"/>
+      <c r="U36" s="12"/>
+    </row>
+    <row r="37" spans="1:21">
+      <c r="A37" s="6">
+        <v>6</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" s="8"/>
+      <c r="D37" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E37" s="9"/>
+      <c r="F37" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="M37" s="12"/>
+      <c r="N37" s="12"/>
+      <c r="O37" s="12"/>
+      <c r="P37" s="12"/>
+      <c r="Q37" s="12"/>
+      <c r="R37" s="12"/>
+      <c r="S37" s="12"/>
+      <c r="T37" s="12"/>
+      <c r="U37" s="12"/>
+    </row>
+    <row r="38" spans="1:21">
+      <c r="A38" s="6"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="12"/>
+      <c r="M38" s="12"/>
+      <c r="N38" s="12"/>
+      <c r="O38" s="12"/>
+      <c r="P38" s="12"/>
+      <c r="Q38" s="12"/>
+      <c r="R38" s="12"/>
+      <c r="S38" s="12"/>
+      <c r="T38" s="12"/>
+      <c r="U38" s="12"/>
+    </row>
+    <row r="39" spans="1:21">
+      <c r="A39" s="6"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
+      <c r="L39" s="12"/>
+      <c r="M39" s="12"/>
+      <c r="N39" s="12"/>
+      <c r="O39" s="12"/>
+      <c r="P39" s="12"/>
+      <c r="Q39" s="12"/>
+      <c r="R39" s="12"/>
+      <c r="S39" s="12"/>
+      <c r="T39" s="12"/>
+      <c r="U39" s="12"/>
+    </row>
+    <row r="40" spans="1:21">
+      <c r="A40" s="6"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="12"/>
+      <c r="M40" s="12"/>
+      <c r="N40" s="12"/>
+      <c r="O40" s="12"/>
+      <c r="P40" s="12"/>
+      <c r="Q40" s="12"/>
+      <c r="R40" s="12"/>
+      <c r="S40" s="12"/>
+      <c r="T40" s="12"/>
+      <c r="U40" s="12"/>
+    </row>
+    <row r="41" spans="1:21">
+      <c r="A41" s="6"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="12"/>
+      <c r="M41" s="12"/>
+      <c r="N41" s="12"/>
+      <c r="O41" s="12"/>
+      <c r="P41" s="12"/>
+      <c r="Q41" s="12"/>
+      <c r="R41" s="12"/>
+      <c r="S41" s="12"/>
+      <c r="T41" s="12"/>
+      <c r="U41" s="12"/>
+    </row>
+    <row r="42" spans="1:21">
+      <c r="A42" s="6"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10"/>
+      <c r="J42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="12"/>
+      <c r="M42" s="12"/>
+      <c r="N42" s="12"/>
+      <c r="O42" s="12"/>
+      <c r="P42" s="12"/>
+      <c r="Q42" s="12"/>
+      <c r="R42" s="12"/>
+      <c r="S42" s="12"/>
+      <c r="T42" s="12"/>
+      <c r="U42" s="12"/>
+    </row>
+    <row r="43" spans="1:21">
+      <c r="A43" s="6"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="12"/>
+      <c r="M43" s="12"/>
+      <c r="N43" s="12"/>
+      <c r="O43" s="12"/>
+      <c r="P43" s="12"/>
+      <c r="Q43" s="12"/>
+      <c r="R43" s="12"/>
+      <c r="S43" s="12"/>
+      <c r="T43" s="12"/>
+      <c r="U43" s="12"/>
+    </row>
+    <row r="44" spans="1:21">
+      <c r="A44" s="6">
+        <v>7</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C44" s="8"/>
+      <c r="D44" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E44" s="9"/>
+      <c r="F44" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
+      <c r="J44" s="10"/>
+      <c r="K44" s="10"/>
+      <c r="L44" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="M44" s="12"/>
+      <c r="N44" s="12"/>
+      <c r="O44" s="12"/>
+      <c r="P44" s="12"/>
+      <c r="Q44" s="12"/>
+      <c r="R44" s="12"/>
+      <c r="S44" s="12"/>
+      <c r="T44" s="12"/>
+      <c r="U44" s="12"/>
+    </row>
+    <row r="45" spans="1:21">
+      <c r="A45" s="6"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
+      <c r="J45" s="10"/>
+      <c r="K45" s="10"/>
+      <c r="L45" s="12"/>
+      <c r="M45" s="12"/>
+      <c r="N45" s="12"/>
+      <c r="O45" s="12"/>
+      <c r="P45" s="12"/>
+      <c r="Q45" s="12"/>
+      <c r="R45" s="12"/>
+      <c r="S45" s="12"/>
+      <c r="T45" s="12"/>
+      <c r="U45" s="12"/>
+    </row>
+    <row r="46" spans="1:21">
+      <c r="A46" s="6"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
+      <c r="J46" s="10"/>
+      <c r="K46" s="10"/>
+      <c r="L46" s="12"/>
+      <c r="M46" s="12"/>
+      <c r="N46" s="12"/>
+      <c r="O46" s="12"/>
+      <c r="P46" s="12"/>
+      <c r="Q46" s="12"/>
+      <c r="R46" s="12"/>
+      <c r="S46" s="12"/>
+      <c r="T46" s="12"/>
+      <c r="U46" s="12"/>
+    </row>
+    <row r="47" spans="1:21">
+      <c r="A47" s="6"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10"/>
+      <c r="J47" s="10"/>
+      <c r="K47" s="10"/>
+      <c r="L47" s="12"/>
+      <c r="M47" s="12"/>
+      <c r="N47" s="12"/>
+      <c r="O47" s="12"/>
+      <c r="P47" s="12"/>
+      <c r="Q47" s="12"/>
+      <c r="R47" s="12"/>
+      <c r="S47" s="12"/>
+      <c r="T47" s="12"/>
+      <c r="U47" s="12"/>
+    </row>
+    <row r="48" spans="1:21">
+      <c r="A48" s="6"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="10"/>
+      <c r="J48" s="10"/>
+      <c r="K48" s="10"/>
+      <c r="L48" s="12"/>
+      <c r="M48" s="12"/>
+      <c r="N48" s="12"/>
+      <c r="O48" s="12"/>
+      <c r="P48" s="12"/>
+      <c r="Q48" s="12"/>
+      <c r="R48" s="12"/>
+      <c r="S48" s="12"/>
+      <c r="T48" s="12"/>
+      <c r="U48" s="12"/>
+    </row>
+    <row r="49" spans="1:21">
+      <c r="A49" s="6"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10"/>
+      <c r="L49" s="12"/>
+      <c r="M49" s="12"/>
+      <c r="N49" s="12"/>
+      <c r="O49" s="12"/>
+      <c r="P49" s="12"/>
+      <c r="Q49" s="12"/>
+      <c r="R49" s="12"/>
+      <c r="S49" s="12"/>
+      <c r="T49" s="12"/>
+      <c r="U49" s="12"/>
+    </row>
+    <row r="50" spans="1:21">
+      <c r="A50" s="6"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10"/>
+      <c r="J50" s="10"/>
+      <c r="K50" s="10"/>
+      <c r="L50" s="12"/>
+      <c r="M50" s="12"/>
+      <c r="N50" s="12"/>
+      <c r="O50" s="12"/>
+      <c r="P50" s="12"/>
+      <c r="Q50" s="12"/>
+      <c r="R50" s="12"/>
+      <c r="S50" s="12"/>
+      <c r="T50" s="12"/>
+      <c r="U50" s="12"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="39">
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="F1:K1"/>
@@ -1952,6 +2989,10 @@
     <mergeCell ref="A2:A8"/>
     <mergeCell ref="A9:A15"/>
     <mergeCell ref="A16:A22"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="A30:A36"/>
+    <mergeCell ref="A37:A43"/>
+    <mergeCell ref="A44:A50"/>
     <mergeCell ref="B2:C8"/>
     <mergeCell ref="D2:E8"/>
     <mergeCell ref="F2:K8"/>
@@ -1964,11 +3005,31 @@
     <mergeCell ref="D16:E22"/>
     <mergeCell ref="F16:K22"/>
     <mergeCell ref="L16:U22"/>
+    <mergeCell ref="B23:C29"/>
+    <mergeCell ref="D23:E29"/>
+    <mergeCell ref="F23:K29"/>
+    <mergeCell ref="L23:U29"/>
+    <mergeCell ref="B30:C36"/>
+    <mergeCell ref="D30:E36"/>
+    <mergeCell ref="F30:K36"/>
+    <mergeCell ref="L30:U36"/>
+    <mergeCell ref="B37:C43"/>
+    <mergeCell ref="D37:E43"/>
+    <mergeCell ref="F37:K43"/>
+    <mergeCell ref="L37:U43"/>
+    <mergeCell ref="B44:C50"/>
+    <mergeCell ref="D44:E50"/>
+    <mergeCell ref="F44:K50"/>
+    <mergeCell ref="L44:U50"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://doi.org/10.1145/3706598.3713164&#10;" tooltip="https://doi.org/10.1145/3706598.3713164&#10;"/>
     <hyperlink ref="B9" r:id="rId2" display="https://www.sciencedirect.com/science/article/pii/S0261517725000032" tooltip="https://www.sciencedirect.com/science/article/pii/S0261517725000032"/>
     <hyperlink ref="B16" r:id="rId3" display="https://doi.org/10.1080/14616688.2025.2532582" tooltip="https://doi.org/10.1080/14616688.2025.2532582"/>
+    <hyperlink ref="B23" r:id="rId4" display="https://dl.acm.org/doi/full/10.1145/3772318.3791068"/>
+    <hyperlink ref="B30" r:id="rId5" display="https://dl.acm.org/doi/10.1145/3706599.3720162#sec-3"/>
+    <hyperlink ref="B37" r:id="rId6" display="https://www.nature.com/articles/s40494-025-01889-3"/>
+    <hyperlink ref="B44" r:id="rId7" display="https://doi.org/10.1145/3700881" tooltip="https://doi.org/10.1145/3700881"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>